<commit_message>
Added sprint 2 story_id to user_stories.xlsx
</commit_message>
<xml_diff>
--- a/Evidence/PP/user_stories.xlsx
+++ b/Evidence/PP/user_stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\PP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61672AE3-06B7-442D-9F0C-D83468A63926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD303E-C473-4567-98F9-D3D531D0DC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="88">
   <si>
     <t>User Story</t>
   </si>
@@ -261,6 +261,42 @@
   </si>
   <si>
     <t>S1-07, 10</t>
+  </si>
+  <si>
+    <t>S2-01</t>
+  </si>
+  <si>
+    <t>S2-02</t>
+  </si>
+  <si>
+    <t>S2-03</t>
+  </si>
+  <si>
+    <t>S2-04</t>
+  </si>
+  <si>
+    <t>S2-05</t>
+  </si>
+  <si>
+    <t>S2-06</t>
+  </si>
+  <si>
+    <t>S2-07</t>
+  </si>
+  <si>
+    <t>S2-08</t>
+  </si>
+  <si>
+    <t>S2-09</t>
+  </si>
+  <si>
+    <t>S2-10</t>
+  </si>
+  <si>
+    <t>S2-11</t>
+  </si>
+  <si>
+    <t>S2-12</t>
   </si>
 </sst>
 </file>
@@ -1161,6 +1197,9 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
+      <c r="J14" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -1190,6 +1229,9 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J15" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -1219,8 +1261,11 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1248,8 +1293,11 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1277,8 +1325,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1310,8 +1361,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -1339,8 +1393,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1368,8 +1425,11 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -1397,8 +1457,11 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1426,8 +1489,11 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -1455,8 +1521,11 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1484,8 +1553,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>25</v>
       </c>
@@ -1514,7 +1586,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
@@ -1543,7 +1615,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
@@ -1572,7 +1644,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>28</v>
       </c>
@@ -1601,7 +1673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>29</v>
       </c>
@@ -1630,7 +1702,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
@@ -1663,7 +1735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
Added PERT predecessors to user_stories.xlsx
</commit_message>
<xml_diff>
--- a/Evidence/PP/user_stories.xlsx
+++ b/Evidence/PP/user_stories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\PP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD303E-C473-4567-98F9-D3D531D0DC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74CF808-5708-4A8C-A58A-7972370C72F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="89">
   <si>
     <t>User Story</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>S2-12</t>
+  </si>
+  <si>
+    <t>S2-02, S2-05</t>
   </si>
 </sst>
 </file>
@@ -1200,6 +1203,9 @@
       <c r="J14" t="s">
         <v>76</v>
       </c>
+      <c r="K14" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -1232,6 +1238,9 @@
       <c r="J15" t="s">
         <v>77</v>
       </c>
+      <c r="K15" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -1264,8 +1273,11 @@
       <c r="J16" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1296,8 +1308,11 @@
       <c r="J17" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1328,8 +1343,11 @@
       <c r="J18" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1364,8 +1382,11 @@
       <c r="J19" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -1396,8 +1417,11 @@
       <c r="J20" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1428,8 +1452,11 @@
       <c r="J21" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -1460,8 +1487,11 @@
       <c r="J22" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1492,8 +1522,11 @@
       <c r="J23" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -1524,8 +1557,11 @@
       <c r="J24" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K24" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1556,8 +1592,11 @@
       <c r="J25" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K25" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>25</v>
       </c>
@@ -1586,7 +1625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
@@ -1615,7 +1654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
@@ -1644,7 +1683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>28</v>
       </c>
@@ -1673,7 +1712,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>29</v>
       </c>
@@ -1702,7 +1741,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
@@ -1735,7 +1774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
Updated user_stories.xlsx added PERT data for Sprint 3 stories
</commit_message>
<xml_diff>
--- a/Evidence/PP/user_stories.xlsx
+++ b/Evidence/PP/user_stories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\PP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C30ECC0-6BAA-4E96-9A50-C521C236B0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFEA418-CCC5-4402-8B70-BF3A1CC2AB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="101">
   <si>
     <t>User Story</t>
   </si>
@@ -300,6 +300,42 @@
   </si>
   <si>
     <t>S2-02, S2-05</t>
+  </si>
+  <si>
+    <t>S3-01</t>
+  </si>
+  <si>
+    <t>S3-02</t>
+  </si>
+  <si>
+    <t>S3-03</t>
+  </si>
+  <si>
+    <t>S3-04</t>
+  </si>
+  <si>
+    <t>S3-05</t>
+  </si>
+  <si>
+    <t>S3-06</t>
+  </si>
+  <si>
+    <t>S3-07</t>
+  </si>
+  <si>
+    <t>S3-08</t>
+  </si>
+  <si>
+    <t>S3-09</t>
+  </si>
+  <si>
+    <t>S3-10</t>
+  </si>
+  <si>
+    <t>S3-11</t>
+  </si>
+  <si>
+    <t>S3-12</t>
   </si>
 </sst>
 </file>
@@ -1624,6 +1660,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J26" t="s">
+        <v>89</v>
+      </c>
+      <c r="K26" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A27" s="3" t="s">
@@ -1653,6 +1695,12 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J27" t="s">
+        <v>90</v>
+      </c>
+      <c r="K27" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A28" s="3" t="s">
@@ -1682,6 +1730,12 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J28" t="s">
+        <v>91</v>
+      </c>
+      <c r="K28" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A29" s="3" t="s">
@@ -1711,6 +1765,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J29" t="s">
+        <v>92</v>
+      </c>
+      <c r="K29" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A30" s="3" t="s">
@@ -1740,6 +1800,12 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J30" t="s">
+        <v>93</v>
+      </c>
+      <c r="K30" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A31" s="3" t="s">
@@ -1773,6 +1839,12 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
+      <c r="J31" t="s">
+        <v>94</v>
+      </c>
+      <c r="K31" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A32" s="3" t="s">
@@ -1802,8 +1874,14 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J32" t="s">
+        <v>95</v>
+      </c>
+      <c r="K32" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A33" s="3" t="s">
         <v>32</v>
       </c>
@@ -1831,8 +1909,14 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J33" t="s">
+        <v>96</v>
+      </c>
+      <c r="K33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
@@ -1860,8 +1944,14 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J34" t="s">
+        <v>97</v>
+      </c>
+      <c r="K34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A35" s="3" t="s">
         <v>34</v>
       </c>
@@ -1889,8 +1979,14 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J35" t="s">
+        <v>98</v>
+      </c>
+      <c r="K35" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A36" s="3" t="s">
         <v>35</v>
       </c>
@@ -1918,8 +2014,14 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J36" t="s">
+        <v>99</v>
+      </c>
+      <c r="K36" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A37" s="3" t="s">
         <v>36</v>
       </c>
@@ -1947,8 +2049,14 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J37" t="s">
+        <v>100</v>
+      </c>
+      <c r="K37" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A38" s="7" t="s">
         <v>12</v>
       </c>
@@ -1977,7 +2085,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A39" s="7" t="s">
         <v>38</v>
       </c>
@@ -2006,7 +2114,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A40" s="7" t="s">
         <v>39</v>
       </c>
@@ -2035,7 +2143,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A41" s="7" t="s">
         <v>40</v>
       </c>
@@ -2064,7 +2172,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
@@ -2093,7 +2201,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A43" s="7" t="s">
         <v>42</v>
       </c>
@@ -2126,7 +2234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A44" s="7" t="s">
         <v>45</v>
       </c>
@@ -2155,7 +2263,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A45" s="7" t="s">
         <v>46</v>
       </c>
@@ -2184,7 +2292,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A46" s="7" t="s">
         <v>47</v>
       </c>
@@ -2213,7 +2321,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A47" s="7" t="s">
         <v>48</v>
       </c>
@@ -2242,7 +2350,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A48" s="7" t="s">
         <v>49</v>
       </c>

</xml_diff>

<commit_message>
Added Story ID for Sprint 4 stories
</commit_message>
<xml_diff>
--- a/Evidence/PP/user_stories.xlsx
+++ b/Evidence/PP/user_stories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\PP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFEA418-CCC5-4402-8B70-BF3A1CC2AB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C77906-5993-4881-ABB1-8CF6F14EA089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="113">
   <si>
     <t>User Story</t>
   </si>
@@ -176,9 +176,6 @@
     <t>As a user, I want to view detailed playback statistics (total listening time, most-played artists) so that I can understand my listening habits.</t>
   </si>
   <si>
-    <t>As a user, I want the player to watch my music folders for file changes so that my library stays accurate without manual scans.</t>
-  </si>
-  <si>
     <t>As a user, I want to export a playlist as a text/CSV file so that I can share it with others or open it somewhere else.</t>
   </si>
   <si>
@@ -336,6 +333,45 @@
   </si>
   <si>
     <t>S3-12</t>
+  </si>
+  <si>
+    <t>As a user, I want to perform advanced searches (e.g., artist:Name or duration&gt;3:00) so that I can filter my library more specifically.</t>
+  </si>
+  <si>
+    <t>S4-01</t>
+  </si>
+  <si>
+    <t>S4-02</t>
+  </si>
+  <si>
+    <t>S4-03</t>
+  </si>
+  <si>
+    <t>S4-04</t>
+  </si>
+  <si>
+    <t>S4-05</t>
+  </si>
+  <si>
+    <t>S4-06</t>
+  </si>
+  <si>
+    <t>S4-07</t>
+  </si>
+  <si>
+    <t>S4-08</t>
+  </si>
+  <si>
+    <t>S4-09</t>
+  </si>
+  <si>
+    <t>S4-10</t>
+  </si>
+  <si>
+    <t>S4-11</t>
+  </si>
+  <si>
+    <t>S4-12</t>
   </si>
 </sst>
 </file>
@@ -760,28 +796,28 @@
         <v>44</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>52</v>
-      </c>
       <c r="F1" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="K1" s="9" t="s">
         <v>58</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.5">
@@ -813,10 +849,10 @@
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.5">
@@ -848,10 +884,10 @@
         <v>5</v>
       </c>
       <c r="J3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" t="s">
         <v>61</v>
-      </c>
-      <c r="K3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.5">
@@ -883,10 +919,10 @@
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.5">
@@ -918,10 +954,10 @@
         <v>2</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.5">
@@ -953,10 +989,10 @@
         <v>3</v>
       </c>
       <c r="J6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.5">
@@ -992,10 +1028,10 @@
         <v>3</v>
       </c>
       <c r="J7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.5">
@@ -1027,10 +1063,10 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.5">
@@ -1062,10 +1098,10 @@
         <v>2</v>
       </c>
       <c r="J9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.5">
@@ -1097,10 +1133,10 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.5">
@@ -1132,10 +1168,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.5">
@@ -1167,10 +1203,10 @@
         <v>3</v>
       </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.5">
@@ -1202,10 +1238,10 @@
         <v>5</v>
       </c>
       <c r="J13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.5">
@@ -1237,10 +1273,10 @@
         <v>3</v>
       </c>
       <c r="J14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.5">
@@ -1272,10 +1308,10 @@
         <v>5</v>
       </c>
       <c r="J15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.5">
@@ -1307,10 +1343,10 @@
         <v>5</v>
       </c>
       <c r="J16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.5">
@@ -1342,10 +1378,10 @@
         <v>2</v>
       </c>
       <c r="J17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.5">
@@ -1377,10 +1413,10 @@
         <v>3</v>
       </c>
       <c r="J18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.5">
@@ -1416,10 +1452,10 @@
         <v>3</v>
       </c>
       <c r="J19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.5">
@@ -1451,10 +1487,10 @@
         <v>3</v>
       </c>
       <c r="J20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.5">
@@ -1486,10 +1522,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.5">
@@ -1521,10 +1557,10 @@
         <v>5</v>
       </c>
       <c r="J22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.5">
@@ -1556,10 +1592,10 @@
         <v>2</v>
       </c>
       <c r="J23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K23" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.5">
@@ -1591,10 +1627,10 @@
         <v>5</v>
       </c>
       <c r="J24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.5">
@@ -1626,10 +1662,10 @@
         <v>3</v>
       </c>
       <c r="J25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.5">
@@ -1661,10 +1697,10 @@
         <v>8</v>
       </c>
       <c r="J26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.5">
@@ -1696,10 +1732,10 @@
         <v>5</v>
       </c>
       <c r="J27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.5">
@@ -1731,10 +1767,10 @@
         <v>5</v>
       </c>
       <c r="J28" t="s">
+        <v>90</v>
+      </c>
+      <c r="K28" t="s">
         <v>91</v>
-      </c>
-      <c r="K28" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.5">
@@ -1766,10 +1802,10 @@
         <v>8</v>
       </c>
       <c r="J29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.5">
@@ -1801,10 +1837,10 @@
         <v>5</v>
       </c>
       <c r="J30" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.5">
@@ -1840,10 +1876,10 @@
         <v>2</v>
       </c>
       <c r="J31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.5">
@@ -1875,10 +1911,10 @@
         <v>8</v>
       </c>
       <c r="J32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.5">
@@ -1910,10 +1946,10 @@
         <v>3</v>
       </c>
       <c r="J33" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.5">
@@ -1945,10 +1981,10 @@
         <v>3</v>
       </c>
       <c r="J34" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.5">
@@ -1980,10 +2016,10 @@
         <v>5</v>
       </c>
       <c r="J35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.5">
@@ -2015,10 +2051,10 @@
         <v>3</v>
       </c>
       <c r="J36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.5">
@@ -2050,10 +2086,10 @@
         <v>3</v>
       </c>
       <c r="J37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.5">
@@ -2084,6 +2120,9 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J38" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A39" s="7" t="s">
@@ -2113,6 +2152,9 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J39" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A40" s="7" t="s">
@@ -2142,6 +2184,9 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J40" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A41" s="7" t="s">
@@ -2171,6 +2216,9 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J41" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A42" s="7" t="s">
@@ -2200,6 +2248,9 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J42" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A43" s="7" t="s">
@@ -2233,6 +2284,9 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
+      <c r="J43" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A44" s="7" t="s">
@@ -2262,6 +2316,9 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J44" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A45" s="7" t="s">
@@ -2291,10 +2348,13 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J45" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A46" s="7" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="B46">
         <v>8</v>
@@ -2320,10 +2380,13 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="J46" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A47" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47">
         <v>5</v>
@@ -2349,10 +2412,13 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
+      <c r="J47" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A48" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48">
         <v>5</v>
@@ -2378,10 +2444,13 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J48" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A49" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49">
         <v>5</v>
@@ -2407,10 +2476,13 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="J49" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A50" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B50">
         <f>SUM(B2:B49)</f>
@@ -2421,9 +2493,9 @@
         <v>175.39</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A51" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B51">
         <f>AVERAGE(B2:B49)</f>
@@ -2434,7 +2506,7 @@
         <v>3.6539583333333332</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A53" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added predecessors for Sprint 4 stories PERT Chart
</commit_message>
<xml_diff>
--- a/Evidence/PP/user_stories.xlsx
+++ b/Evidence/PP/user_stories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\PP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9A1033-2741-4590-9F9C-9D7E53BE9C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DEDDCAE-C1D3-4445-A9AF-9870422FE305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="113">
   <si>
     <t>User Story</t>
   </si>
@@ -2123,6 +2123,9 @@
       <c r="J38" t="s">
         <v>101</v>
       </c>
+      <c r="K38" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A39" s="7" t="s">
@@ -2155,6 +2158,9 @@
       <c r="J39" t="s">
         <v>102</v>
       </c>
+      <c r="K39" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A40" s="7" t="s">
@@ -2187,6 +2193,9 @@
       <c r="J40" t="s">
         <v>103</v>
       </c>
+      <c r="K40" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A41" s="7" t="s">
@@ -2219,6 +2228,9 @@
       <c r="J41" t="s">
         <v>104</v>
       </c>
+      <c r="K41" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A42" s="7" t="s">
@@ -2251,6 +2263,9 @@
       <c r="J42" t="s">
         <v>105</v>
       </c>
+      <c r="K42" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A43" s="7" t="s">
@@ -2287,6 +2302,9 @@
       <c r="J43" t="s">
         <v>106</v>
       </c>
+      <c r="K43" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A44" s="7" t="s">
@@ -2319,6 +2337,9 @@
       <c r="J44" t="s">
         <v>107</v>
       </c>
+      <c r="K44" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A45" s="7" t="s">
@@ -2351,6 +2372,9 @@
       <c r="J45" t="s">
         <v>108</v>
       </c>
+      <c r="K45" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A46" s="7" t="s">
@@ -2383,6 +2407,9 @@
       <c r="J46" t="s">
         <v>109</v>
       </c>
+      <c r="K46" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A47" s="7" t="s">
@@ -2415,6 +2442,9 @@
       <c r="J47" t="s">
         <v>110</v>
       </c>
+      <c r="K47" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A48" s="7" t="s">
@@ -2447,8 +2477,11 @@
       <c r="J48" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.5">
+      <c r="K48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A49" s="7" t="s">
         <v>49</v>
       </c>
@@ -2479,8 +2512,11 @@
       <c r="J49" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.5">
+      <c r="K49" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A50" s="9" t="s">
         <v>52</v>
       </c>
@@ -2493,7 +2529,7 @@
         <v>175.39</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A51" s="9" t="s">
         <v>53</v>
       </c>
@@ -2506,7 +2542,7 @@
         <v>3.6539583333333332</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.5">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A53" s="1"/>
     </row>
   </sheetData>

</xml_diff>